<commit_message>
SFBS data update 5/19
</commit_message>
<xml_diff>
--- a/data_raw/smelt/SFBS_2026.xlsx
+++ b/data_raw/smelt/SFBS_2026.xlsx
@@ -10502,4 +10502,10 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{6dd02d64-b7f3-43f7-a145-cfd68d338edf}" enabled="1" method="Standard" siteId="{0693b5ba-4b18-4d7b-9341-f32f400a5494}" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>